<commit_message>
fixed time and room dropdown, added selected slot when clicking the modules on the conflict section, added new test files
</commit_message>
<xml_diff>
--- a/ITP Programming App 2/Data/Excel Test Files/realistic_with_conflicts.xlsx
+++ b/ITP Programming App 2/Data/Excel Test Files/realistic_with_conflicts.xlsx
@@ -21136,29 +21136,17 @@
       </c>
       <c r="F2" s="10" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="G2" s="10" t="n"/>
       <c r="H2" s="10" t="n"/>
-      <c r="I2" s="10" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="J2" s="10" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="K2" s="10" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
+      <c r="I2" s="10" t="n"/>
+      <c r="J2" s="10" t="n"/>
+      <c r="K2" s="10" t="n"/>
       <c r="L2" s="10" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="M2" s="10" t="inlineStr">
@@ -21168,17 +21156,9 @@
       </c>
       <c r="N2" s="89" t="n"/>
       <c r="O2" s="89" t="n"/>
-      <c r="P2" s="89" t="inlineStr">
-        <is>
-          <t>CONFLICT (Student Group): Clashes with REQ-ACC-ACC1025-LEC-01. ACC Y1 P1 is double-booked at Thursday 09:00-11:00.</t>
-        </is>
-      </c>
+      <c r="P2" s="89" t="n"/>
       <c r="Q2" s="89" t="n"/>
-      <c r="R2" s="148" t="inlineStr">
-        <is>
-          <t>Intentionally added time conflict for testing (student group clash with REQ-ACC-ACC1025-LEC-01).</t>
-        </is>
-      </c>
+      <c r="R2" s="148" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="56" t="inlineStr">
@@ -21348,29 +21328,17 @@
       </c>
       <c r="F6" s="24" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="G6" s="24" t="n"/>
       <c r="H6" s="24" t="n"/>
-      <c r="I6" s="24" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="J6" s="24" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="K6" s="24" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
+      <c r="I6" s="24" t="n"/>
+      <c r="J6" s="24" t="n"/>
+      <c r="K6" s="24" t="n"/>
       <c r="L6" s="24" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="M6" s="24" t="inlineStr">
@@ -21380,17 +21348,9 @@
       </c>
       <c r="N6" s="93" t="n"/>
       <c r="O6" s="93" t="n"/>
-      <c r="P6" s="93" t="inlineStr">
-        <is>
-          <t>CONFLICT (Student Group): Clashes with REQ-ACC-ACC1023-LEC-01. ACC Y1 P1 is double-booked at Thursday 09:00-11:00.</t>
-        </is>
-      </c>
+      <c r="P6" s="93" t="n"/>
       <c r="Q6" s="93" t="n"/>
-      <c r="R6" s="152" t="inlineStr">
-        <is>
-          <t>Intentionally added time conflict for testing (student group clash with REQ-ACC-ACC1023-LEC-01).</t>
-        </is>
-      </c>
+      <c r="R6" s="152" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="60" t="inlineStr">
@@ -22074,13 +22034,13 @@
       <c r="O20" s="96" t="n"/>
       <c r="P20" s="96" t="inlineStr">
         <is>
-          <t>CONFLICT (Lecturer): Clashes with REQ-ASE-ASE3106-LEC-01. EMP2961 is double-booked at Monday 09:00-11:00.</t>
+          <t>CONFLICT: same time as REQ-ASE-ASE3106-LEC-01 (Monday 09:00-11:00).</t>
         </is>
       </c>
       <c r="Q20" s="96" t="n"/>
       <c r="R20" s="155" t="inlineStr">
         <is>
-          <t>Intentionally added time conflict for testing (lecturer clash with REQ-ASE-ASE3106-LEC-01).</t>
+          <t>Same time as REQ-ASE-ASE3106-LEC-01.</t>
         </is>
       </c>
     </row>
@@ -22190,13 +22150,13 @@
       <c r="O22" s="98" t="n"/>
       <c r="P22" s="98" t="inlineStr">
         <is>
-          <t>CONFLICT (Lecturer): Clashes with REQ-ASE-ASE2210-LEC-01. EMP2961 is double-booked at Monday 09:00-11:00.</t>
+          <t>CONFLICT: same time as REQ-ASE-ASE2210-LEC-01 (Monday 09:00-11:00).</t>
         </is>
       </c>
       <c r="Q22" s="98" t="n"/>
       <c r="R22" s="157" t="inlineStr">
         <is>
-          <t>Intentionally added time conflict for testing (lecturer clash with REQ-ASE-ASE2210-LEC-01).</t>
+          <t>Same time as REQ-ASE-ASE2210-LEC-01.</t>
         </is>
       </c>
     </row>
@@ -22354,13 +22314,13 @@
       <c r="O25" s="90" t="n"/>
       <c r="P25" s="90" t="inlineStr">
         <is>
-          <t>CONFLICT (Venue): Clashes with REQ-ATM-ATM3302-TUT-02. ATM Seminar Room is double-booked at Monday 11:00-13:00.</t>
+          <t>CONFLICT: same time as REQ-ATM-ATM3302-TUT-02 (Monday 11:00-13:00).</t>
         </is>
       </c>
       <c r="Q25" s="90" t="n"/>
       <c r="R25" s="149" t="inlineStr">
         <is>
-          <t>Intentionally added time conflict for testing (venue clash with REQ-ATM-ATM3302-TUT-02).</t>
+          <t>Same time as REQ-ATM-ATM3302-TUT-02.</t>
         </is>
       </c>
     </row>
@@ -22806,13 +22766,13 @@
       <c r="O34" s="99" t="n"/>
       <c r="P34" s="99" t="inlineStr">
         <is>
-          <t>CONFLICT (Venue): Clashes with REQ-ATM-ATM1104-TUT-02. ATM Seminar Room is double-booked at Monday 11:00-13:00.</t>
+          <t>CONFLICT: same time as REQ-ATM-ATM1104-TUT-02 (Monday 11:00-13:00).</t>
         </is>
       </c>
       <c r="Q34" s="99" t="n"/>
       <c r="R34" s="158" t="inlineStr">
         <is>
-          <t>Intentionally added time conflict for testing (venue clash with REQ-ATM-ATM1104-TUT-02).</t>
+          <t>Same time as REQ-ATM-ATM1104-TUT-02.</t>
         </is>
       </c>
     </row>
@@ -22840,17 +22800,29 @@
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G35" s="10" t="n"/>
       <c r="H35" s="10" t="n"/>
-      <c r="I35" s="10" t="n"/>
-      <c r="J35" s="10" t="n"/>
-      <c r="K35" s="10" t="n"/>
+      <c r="I35" s="10" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="J35" s="10" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="K35" s="10" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
       <c r="L35" s="10" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="M35" s="10" t="inlineStr">
@@ -22860,9 +22832,17 @@
       </c>
       <c r="N35" s="89" t="n"/>
       <c r="O35" s="89" t="n"/>
-      <c r="P35" s="89" t="n"/>
+      <c r="P35" s="89" t="inlineStr">
+        <is>
+          <t>CONFLICT: same time as REQ-BAC-BAC2005-LEC-01 (Friday 09:00-11:00).</t>
+        </is>
+      </c>
       <c r="Q35" s="89" t="n"/>
-      <c r="R35" s="148" t="n"/>
+      <c r="R35" s="148" t="inlineStr">
+        <is>
+          <t>Same time as REQ-BAC-BAC2005-LEC-01.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="56" t="inlineStr">
@@ -23032,17 +23012,29 @@
       </c>
       <c r="F39" s="24" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G39" s="24" t="n"/>
       <c r="H39" s="24" t="n"/>
-      <c r="I39" s="24" t="n"/>
-      <c r="J39" s="24" t="n"/>
-      <c r="K39" s="24" t="n"/>
+      <c r="I39" s="24" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="J39" s="24" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="K39" s="24" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
       <c r="L39" s="24" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="M39" s="24" t="inlineStr">
@@ -23052,9 +23044,17 @@
       </c>
       <c r="N39" s="93" t="n"/>
       <c r="O39" s="93" t="n"/>
-      <c r="P39" s="93" t="n"/>
+      <c r="P39" s="93" t="inlineStr">
+        <is>
+          <t>CONFLICT: same time as REQ-BAC-BAC2001-LEC-01 (Friday 09:00-11:00).</t>
+        </is>
+      </c>
       <c r="Q39" s="93" t="n"/>
-      <c r="R39" s="152" t="n"/>
+      <c r="R39" s="152" t="inlineStr">
+        <is>
+          <t>Same time as REQ-BAC-BAC2001-LEC-01.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="60" t="inlineStr">
@@ -24952,29 +24952,17 @@
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="G79" s="10" t="n"/>
       <c r="H79" s="10" t="n"/>
-      <c r="I79" s="10" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="J79" s="10" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="K79" s="10" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
+      <c r="I79" s="10" t="n"/>
+      <c r="J79" s="10" t="n"/>
+      <c r="K79" s="10" t="n"/>
       <c r="L79" s="10" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="M79" s="10" t="inlineStr">
@@ -24984,17 +24972,9 @@
       </c>
       <c r="N79" s="89" t="n"/>
       <c r="O79" s="89" t="n"/>
-      <c r="P79" s="89" t="inlineStr">
-        <is>
-          <t>CONFLICT (Lecturer): Clashes with REQ-DSC-DSC3302-LEC-01. EMP3183 is double-booked at Tuesday 09:00-11:00.</t>
-        </is>
-      </c>
+      <c r="P79" s="89" t="n"/>
       <c r="Q79" s="89" t="n"/>
-      <c r="R79" s="148" t="inlineStr">
-        <is>
-          <t>Intentionally added time conflict for testing (lecturer clash with REQ-DSC-DSC3302-LEC-01).</t>
-        </is>
-      </c>
+      <c r="R79" s="148" t="n"/>
     </row>
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="56" t="inlineStr">
@@ -25308,29 +25288,17 @@
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="G86" s="34" t="n"/>
       <c r="H86" s="34" t="n"/>
-      <c r="I86" s="34" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="J86" s="34" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="K86" s="34" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
+      <c r="I86" s="34" t="n"/>
+      <c r="J86" s="34" t="n"/>
+      <c r="K86" s="34" t="n"/>
       <c r="L86" s="34" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="M86" s="34" t="inlineStr">
@@ -25340,17 +25308,9 @@
       </c>
       <c r="N86" s="96" t="n"/>
       <c r="O86" s="96" t="n"/>
-      <c r="P86" s="96" t="inlineStr">
-        <is>
-          <t>CONFLICT (Lecturer): Clashes with REQ-DSC-DSC2203-LEC-01. EMP3183 is double-booked at Tuesday 09:00-11:00.</t>
-        </is>
-      </c>
+      <c r="P86" s="96" t="n"/>
       <c r="Q86" s="96" t="n"/>
-      <c r="R86" s="155" t="inlineStr">
-        <is>
-          <t>Intentionally added time conflict for testing (lecturer clash with REQ-DSC-DSC2203-LEC-01).</t>
-        </is>
-      </c>
+      <c r="R86" s="155" t="n"/>
     </row>
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="63" t="inlineStr">

</xml_diff>